<commit_message>
Add carousel-homepage block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/carousel-homepage/carousel-homepage.css
- blocks/carousel-homepage/carousel-homepage.js
- blocks/carousel-homepage/metadata.json
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/parsers/carousel-homepage.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-carousel","columns-news","columns-news","columns-news","cards-feature","cards-feature","cards-feature","tabs-resources","columns-contact"]</t>
+    <t>["carousel-homepage","columns-news","columns-news","columns-news","cards-feature","cards-feature","cards-feature","tabs-resources","columns-contact"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-23T19:06:52.883Z</t>
+    <t>2026-04-23T19:33:39.334Z</t>
   </si>
   <si>
     <t>WorkSafeNB | WorkSafeNB</t>

</xml_diff>